<commit_message>
chinh sua cv 1 xiu
</commit_message>
<xml_diff>
--- a/BA Project/RACI-Matrix-Template.xlsx
+++ b/BA Project/RACI-Matrix-Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\usb\G\Learning\others\Portfolio\my_portfolio\BA Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3572C24-3583-47A3-B0EC-207FE5982F9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B96E6AB-83CF-4BFC-B68D-18F9FB54BE4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RACI Matrix Example" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="60">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -648,12 +648,24 @@
   <si>
     <t>User</t>
   </si>
+  <si>
+    <t>R = Responsible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A = Accountable </t>
+  </si>
+  <si>
+    <t>C = Consulted</t>
+  </si>
+  <si>
+    <t>I = Informed</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -789,11 +801,17 @@
     </font>
     <font>
       <b/>
-      <sz val="16"/>
+      <sz val="11"/>
+      <color theme="2"/>
+      <name val="Montserrat"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <name val="Montserrat"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -869,6 +887,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF132591"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF39B836"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1216,7 +1252,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1258,18 +1294,96 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1279,6 +1393,30 @@
     <xf numFmtId="0" fontId="10" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1288,124 +1426,28 @@
     <xf numFmtId="0" fontId="15" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="7" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1414,29 +1456,42 @@
     <xf numFmtId="0" fontId="22" fillId="7" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="22" fillId="11" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="36">
+  <dxfs count="12">
     <dxf>
       <fill>
         <patternFill>
@@ -1521,183 +1576,15 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD41628"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF132591"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD41628"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF39B836"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF132591"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD41628"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEBED"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF132591"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDFDEFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEBED"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF132591"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDFDEFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC5EDEC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEBED"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF132591"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDFDEFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC5EDEC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEBED"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFE9BF"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{FD192230-E4A4-4724-87CC-1E2186F3AAE1}"/>
   </tableStyles>
   <colors>
     <mruColors>
+      <color rgb="FFCEF4FF"/>
+      <color rgb="FF132591"/>
       <color rgb="FF39B836"/>
-      <color rgb="FF132591"/>
-      <color rgb="FFCEF4FF"/>
       <color rgb="FFD41628"/>
       <color rgb="FF30206B"/>
     </mruColors>
@@ -2200,13 +2087,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:24" ht="52.05" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
     </row>
     <row r="2" spans="2:24" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B2" s="3" t="s">
@@ -2217,14 +2104,14 @@
       <c r="F2" s="3"/>
     </row>
     <row r="3" spans="2:24" s="11" customFormat="1" ht="76.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="46" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
-      <c r="G3" s="20"/>
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="46"/>
+      <c r="F3" s="46"/>
+      <c r="G3" s="46"/>
       <c r="J3" s="12"/>
       <c r="K3" s="12"/>
       <c r="L3" s="12"/>
@@ -2251,277 +2138,277 @@
       <c r="Q4" s="12"/>
     </row>
     <row r="5" spans="2:24" ht="67.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B5" s="41" t="s">
+      <c r="B5" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="41" t="s">
+      <c r="C5" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="41" t="s">
+      <c r="D5" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="E5" s="41" t="s">
+      <c r="E5" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="F5" s="41" t="s">
+      <c r="F5" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="G5" s="41" t="s">
+      <c r="G5" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="H5" s="41" t="s">
+      <c r="H5" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="K5" s="21" t="s">
+      <c r="K5" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="L5" s="22"/>
-      <c r="M5" s="22"/>
-      <c r="N5" s="22"/>
-      <c r="O5" s="22"/>
-      <c r="P5" s="23"/>
+      <c r="L5" s="48"/>
+      <c r="M5" s="48"/>
+      <c r="N5" s="48"/>
+      <c r="O5" s="48"/>
+      <c r="P5" s="49"/>
     </row>
     <row r="6" spans="2:24" ht="49.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B6" s="53" t="s">
+      <c r="B6" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="C6" s="54" t="s">
+      <c r="C6" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="54" t="s">
+      <c r="D6" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="54" t="s">
+      <c r="E6" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="F6" s="54" t="s">
+      <c r="F6" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="G6" s="54" t="s">
+      <c r="G6" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="H6" s="54" t="s">
+      <c r="H6" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="K6" s="55" t="s">
+      <c r="K6" s="40" t="s">
         <v>49</v>
       </c>
-      <c r="L6" s="55"/>
-      <c r="M6" s="55"/>
-      <c r="N6" s="56" t="s">
+      <c r="L6" s="40"/>
+      <c r="M6" s="40"/>
+      <c r="N6" s="42" t="s">
         <v>50</v>
       </c>
-      <c r="O6" s="56"/>
-      <c r="P6" s="56"/>
+      <c r="O6" s="42"/>
+      <c r="P6" s="42"/>
     </row>
     <row r="7" spans="2:24" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B7" s="53" t="s">
+      <c r="B7" s="29" t="s">
         <v>35</v>
       </c>
-      <c r="C7" s="54" t="s">
+      <c r="C7" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="D7" s="54" t="s">
+      <c r="D7" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="E7" s="54" t="s">
+      <c r="E7" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="F7" s="54" t="s">
+      <c r="F7" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="G7" s="54" t="s">
+      <c r="G7" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="H7" s="54" t="s">
+      <c r="H7" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="K7" s="57"/>
-      <c r="L7" s="57"/>
-      <c r="M7" s="57"/>
-      <c r="N7" s="58"/>
-      <c r="O7" s="58"/>
-      <c r="P7" s="58"/>
+      <c r="K7" s="41"/>
+      <c r="L7" s="41"/>
+      <c r="M7" s="41"/>
+      <c r="N7" s="43"/>
+      <c r="O7" s="43"/>
+      <c r="P7" s="43"/>
     </row>
     <row r="8" spans="2:24" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B8" s="53" t="s">
+      <c r="B8" s="29" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="54" t="s">
+      <c r="C8" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="D8" s="54" t="s">
+      <c r="D8" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="E8" s="54" t="s">
+      <c r="E8" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="F8" s="54" t="s">
+      <c r="F8" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="G8" s="54" t="s">
+      <c r="G8" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="H8" s="54" t="s">
+      <c r="H8" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="K8" s="57"/>
-      <c r="L8" s="57"/>
-      <c r="M8" s="57"/>
-      <c r="N8" s="58"/>
-      <c r="O8" s="58"/>
-      <c r="P8" s="58"/>
+      <c r="K8" s="41"/>
+      <c r="L8" s="41"/>
+      <c r="M8" s="41"/>
+      <c r="N8" s="43"/>
+      <c r="O8" s="43"/>
+      <c r="P8" s="43"/>
     </row>
     <row r="9" spans="2:24" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B9" s="53" t="s">
+      <c r="B9" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="C9" s="54" t="s">
+      <c r="C9" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="D9" s="54" t="s">
+      <c r="D9" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="E9" s="54" t="s">
+      <c r="E9" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="F9" s="54" t="s">
+      <c r="F9" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="G9" s="54" t="s">
+      <c r="G9" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="H9" s="54" t="s">
+      <c r="H9" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="K9" s="57"/>
-      <c r="L9" s="57"/>
-      <c r="M9" s="57"/>
-      <c r="N9" s="58"/>
-      <c r="O9" s="58"/>
-      <c r="P9" s="58"/>
+      <c r="K9" s="41"/>
+      <c r="L9" s="41"/>
+      <c r="M9" s="41"/>
+      <c r="N9" s="43"/>
+      <c r="O9" s="43"/>
+      <c r="P9" s="43"/>
     </row>
     <row r="10" spans="2:24" ht="38.4" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B10" s="53" t="s">
+      <c r="B10" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="C10" s="54" t="s">
+      <c r="C10" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="D10" s="61" t="s">
+      <c r="D10" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="E10" s="54" t="s">
+      <c r="E10" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="F10" s="54" t="s">
+      <c r="F10" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="G10" s="54" t="s">
+      <c r="G10" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="H10" s="54" t="s">
+      <c r="H10" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="K10" s="59" t="s">
+      <c r="K10" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="L10" s="59"/>
-      <c r="M10" s="59"/>
-      <c r="N10" s="60" t="s">
+      <c r="L10" s="38"/>
+      <c r="M10" s="38"/>
+      <c r="N10" s="39" t="s">
         <v>52</v>
       </c>
-      <c r="O10" s="60"/>
-      <c r="P10" s="60"/>
+      <c r="O10" s="39"/>
+      <c r="P10" s="39"/>
     </row>
     <row r="11" spans="2:24" ht="30.6" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B11" s="53" t="s">
+      <c r="B11" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="54" t="s">
+      <c r="C11" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="D11" s="54" t="s">
+      <c r="D11" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="E11" s="54" t="s">
+      <c r="E11" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="F11" s="54" t="s">
+      <c r="F11" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="G11" s="54" t="s">
+      <c r="G11" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="H11" s="54" t="s">
+      <c r="H11" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="K11" s="59"/>
-      <c r="L11" s="59"/>
-      <c r="M11" s="59"/>
-      <c r="N11" s="60"/>
-      <c r="O11" s="60"/>
-      <c r="P11" s="60"/>
+      <c r="K11" s="38"/>
+      <c r="L11" s="38"/>
+      <c r="M11" s="38"/>
+      <c r="N11" s="39"/>
+      <c r="O11" s="39"/>
+      <c r="P11" s="39"/>
     </row>
     <row r="12" spans="2:24" ht="43.8" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B12" s="53" t="s">
+      <c r="B12" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="C12" s="54" t="s">
+      <c r="C12" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="D12" s="54" t="s">
+      <c r="D12" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="E12" s="54" t="s">
+      <c r="E12" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="F12" s="54" t="s">
+      <c r="F12" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="G12" s="54" t="s">
+      <c r="G12" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="H12" s="54" t="s">
+      <c r="H12" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="K12" s="59"/>
-      <c r="L12" s="59"/>
-      <c r="M12" s="59"/>
-      <c r="N12" s="60"/>
-      <c r="O12" s="60"/>
-      <c r="P12" s="60"/>
+      <c r="K12" s="38"/>
+      <c r="L12" s="38"/>
+      <c r="M12" s="38"/>
+      <c r="N12" s="39"/>
+      <c r="O12" s="39"/>
+      <c r="P12" s="39"/>
     </row>
     <row r="13" spans="2:24" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="53" t="s">
+      <c r="B13" s="29" t="s">
         <v>41</v>
       </c>
-      <c r="C13" s="54" t="s">
+      <c r="C13" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="D13" s="54" t="s">
+      <c r="D13" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="E13" s="54" t="s">
+      <c r="E13" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="F13" s="54" t="s">
+      <c r="F13" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="G13" s="54" t="s">
+      <c r="G13" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="H13" s="54" t="s">
+      <c r="H13" s="30" t="s">
         <v>5</v>
       </c>
       <c r="I13" s="4"/>
       <c r="J13" s="10"/>
-      <c r="K13" s="59"/>
-      <c r="L13" s="59"/>
-      <c r="M13" s="59"/>
-      <c r="N13" s="60"/>
-      <c r="O13" s="60"/>
-      <c r="P13" s="60"/>
+      <c r="K13" s="38"/>
+      <c r="L13" s="38"/>
+      <c r="M13" s="38"/>
+      <c r="N13" s="39"/>
+      <c r="O13" s="39"/>
+      <c r="P13" s="39"/>
       <c r="Q13" s="10"/>
       <c r="R13" s="4"/>
       <c r="S13" s="4"/>
@@ -2532,35 +2419,35 @@
       <c r="X13" s="4"/>
     </row>
     <row r="14" spans="2:24" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="53" t="s">
+      <c r="B14" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C14" s="54" t="s">
+      <c r="C14" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="D14" s="54" t="s">
+      <c r="D14" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="E14" s="54" t="s">
+      <c r="E14" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="F14" s="54" t="s">
+      <c r="F14" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="G14" s="54" t="s">
+      <c r="G14" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="H14" s="54" t="s">
+      <c r="H14" s="30" t="s">
         <v>4</v>
       </c>
       <c r="I14" s="4"/>
       <c r="J14" s="10"/>
-      <c r="K14" s="59"/>
-      <c r="L14" s="59"/>
-      <c r="M14" s="59"/>
-      <c r="N14" s="60"/>
-      <c r="O14" s="60"/>
-      <c r="P14" s="60"/>
+      <c r="K14" s="38"/>
+      <c r="L14" s="38"/>
+      <c r="M14" s="38"/>
+      <c r="N14" s="39"/>
+      <c r="O14" s="39"/>
+      <c r="P14" s="39"/>
       <c r="Q14" s="10"/>
       <c r="R14" s="4"/>
       <c r="S14" s="4"/>
@@ -2571,35 +2458,35 @@
       <c r="X14" s="4"/>
     </row>
     <row r="15" spans="2:24" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="53" t="s">
+      <c r="B15" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="C15" s="54" t="s">
+      <c r="C15" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="D15" s="54" t="s">
+      <c r="D15" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="E15" s="54" t="s">
+      <c r="E15" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="F15" s="54" t="s">
+      <c r="F15" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="G15" s="54" t="s">
+      <c r="G15" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="H15" s="54" t="s">
+      <c r="H15" s="30" t="s">
         <v>5</v>
       </c>
       <c r="I15" s="4"/>
       <c r="J15" s="10"/>
-      <c r="K15" s="59"/>
-      <c r="L15" s="59"/>
-      <c r="M15" s="59"/>
-      <c r="N15" s="60"/>
-      <c r="O15" s="60"/>
-      <c r="P15" s="60"/>
+      <c r="K15" s="38"/>
+      <c r="L15" s="38"/>
+      <c r="M15" s="38"/>
+      <c r="N15" s="39"/>
+      <c r="O15" s="39"/>
+      <c r="P15" s="39"/>
       <c r="Q15" s="10"/>
       <c r="R15" s="4"/>
       <c r="S15" s="4"/>
@@ -2610,12 +2497,12 @@
       <c r="X15" s="4"/>
     </row>
     <row r="16" spans="2:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="K16" s="59"/>
-      <c r="L16" s="59"/>
-      <c r="M16" s="59"/>
-      <c r="N16" s="60"/>
-      <c r="O16" s="60"/>
-      <c r="P16" s="60"/>
+      <c r="K16" s="38"/>
+      <c r="L16" s="38"/>
+      <c r="M16" s="38"/>
+      <c r="N16" s="39"/>
+      <c r="O16" s="39"/>
+      <c r="P16" s="39"/>
     </row>
     <row r="17" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
     <row r="18" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
@@ -3633,12 +3520,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:24" ht="52.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
     </row>
     <row r="2" spans="2:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B2" s="3" t="s">
@@ -3649,15 +3536,15 @@
       <c r="E2" s="3"/>
     </row>
     <row r="3" spans="2:24" s="11" customFormat="1" ht="100.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="24" t="s">
+      <c r="B3" s="58" t="s">
         <v>44</v>
       </c>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="24"/>
-      <c r="F3" s="24"/>
-      <c r="G3" s="24"/>
-      <c r="H3" s="24"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="58"/>
+      <c r="G3" s="58"/>
+      <c r="H3" s="58"/>
       <c r="J3" s="12"/>
       <c r="K3" s="12"/>
       <c r="L3" s="12"/>
@@ -3668,307 +3555,307 @@
       <c r="Q3" s="12"/>
     </row>
     <row r="4" spans="2:24" ht="67.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B4" s="41" t="s">
+      <c r="B4" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="C4" s="42" t="s">
+      <c r="C4" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="D4" s="43" t="s">
+      <c r="D4" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="E4" s="43" t="s">
+      <c r="E4" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="43" t="s">
+      <c r="F4" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="43" t="s">
+      <c r="G4" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="H4" s="43" t="s">
+      <c r="H4" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="K4" s="21" t="s">
+      <c r="K4" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="L4" s="22"/>
-      <c r="M4" s="22"/>
-      <c r="N4" s="22"/>
-      <c r="O4" s="22"/>
-      <c r="P4" s="23"/>
+      <c r="L4" s="48"/>
+      <c r="M4" s="48"/>
+      <c r="N4" s="48"/>
+      <c r="O4" s="48"/>
+      <c r="P4" s="49"/>
     </row>
     <row r="5" spans="2:24" ht="67.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B5" s="44" t="s">
+      <c r="B5" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="C5" s="45" t="s">
+      <c r="C5" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="46" t="s">
+      <c r="D5" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="E5" s="46" t="s">
+      <c r="E5" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="F5" s="46" t="s">
+      <c r="F5" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="G5" s="46" t="s">
+      <c r="G5" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="H5" s="46" t="s">
+      <c r="H5" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="K5" s="25" t="s">
+      <c r="K5" s="59" t="s">
         <v>45</v>
       </c>
-      <c r="L5" s="26"/>
-      <c r="M5" s="26"/>
-      <c r="N5" s="27" t="s">
+      <c r="L5" s="60"/>
+      <c r="M5" s="60"/>
+      <c r="N5" s="63" t="s">
         <v>46</v>
       </c>
-      <c r="O5" s="27"/>
-      <c r="P5" s="28"/>
+      <c r="O5" s="63"/>
+      <c r="P5" s="64"/>
     </row>
     <row r="6" spans="2:24" ht="67.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B6" s="47" t="s">
+      <c r="B6" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="C6" s="48" t="s">
+      <c r="C6" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="49" t="s">
+      <c r="D6" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="E6" s="49" t="s">
+      <c r="E6" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="F6" s="49" t="s">
+      <c r="F6" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="G6" s="49" t="s">
+      <c r="G6" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="H6" s="49" t="s">
+      <c r="H6" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="K6" s="29"/>
-      <c r="L6" s="30"/>
-      <c r="M6" s="30"/>
-      <c r="N6" s="31"/>
-      <c r="O6" s="31"/>
-      <c r="P6" s="32"/>
+      <c r="K6" s="61"/>
+      <c r="L6" s="62"/>
+      <c r="M6" s="62"/>
+      <c r="N6" s="65"/>
+      <c r="O6" s="65"/>
+      <c r="P6" s="66"/>
     </row>
     <row r="7" spans="2:24" ht="67.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B7" s="47" t="s">
+      <c r="B7" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="C7" s="48" t="s">
+      <c r="C7" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="D7" s="49" t="s">
+      <c r="D7" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="E7" s="49" t="s">
+      <c r="E7" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="F7" s="49" t="s">
+      <c r="F7" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="G7" s="49" t="s">
+      <c r="G7" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="H7" s="49" t="s">
+      <c r="H7" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="K7" s="29"/>
-      <c r="L7" s="30"/>
-      <c r="M7" s="30"/>
-      <c r="N7" s="31"/>
-      <c r="O7" s="31"/>
-      <c r="P7" s="32"/>
+      <c r="K7" s="61"/>
+      <c r="L7" s="62"/>
+      <c r="M7" s="62"/>
+      <c r="N7" s="65"/>
+      <c r="O7" s="65"/>
+      <c r="P7" s="66"/>
     </row>
     <row r="8" spans="2:24" ht="67.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B8" s="47" t="s">
+      <c r="B8" s="23" t="s">
         <v>37</v>
       </c>
-      <c r="C8" s="48" t="s">
+      <c r="C8" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="D8" s="49" t="s">
+      <c r="D8" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="E8" s="49" t="s">
+      <c r="E8" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="F8" s="49" t="s">
+      <c r="F8" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="G8" s="49" t="s">
+      <c r="G8" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="H8" s="49" t="s">
+      <c r="H8" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="K8" s="33" t="s">
+      <c r="K8" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="L8" s="34"/>
-      <c r="M8" s="34"/>
-      <c r="N8" s="35" t="s">
+      <c r="L8" s="51"/>
+      <c r="M8" s="51"/>
+      <c r="N8" s="54" t="s">
         <v>48</v>
       </c>
-      <c r="O8" s="35"/>
-      <c r="P8" s="36"/>
+      <c r="O8" s="54"/>
+      <c r="P8" s="55"/>
     </row>
     <row r="9" spans="2:24" ht="67.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B9" s="47" t="s">
+      <c r="B9" s="23" t="s">
         <v>38</v>
       </c>
-      <c r="C9" s="48" t="s">
+      <c r="C9" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="D9" s="49" t="s">
+      <c r="D9" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="E9" s="49" t="s">
+      <c r="E9" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="F9" s="49" t="s">
+      <c r="F9" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="G9" s="49" t="s">
+      <c r="G9" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="H9" s="49" t="s">
+      <c r="H9" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="K9" s="33"/>
-      <c r="L9" s="34"/>
-      <c r="M9" s="34"/>
-      <c r="N9" s="35"/>
-      <c r="O9" s="35"/>
-      <c r="P9" s="36"/>
+      <c r="K9" s="50"/>
+      <c r="L9" s="51"/>
+      <c r="M9" s="51"/>
+      <c r="N9" s="54"/>
+      <c r="O9" s="54"/>
+      <c r="P9" s="55"/>
     </row>
     <row r="10" spans="2:24" ht="67.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B10" s="47" t="s">
+      <c r="B10" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="C10" s="48" t="s">
+      <c r="C10" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="D10" s="49" t="s">
+      <c r="D10" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="E10" s="49" t="s">
+      <c r="E10" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="F10" s="49" t="s">
+      <c r="F10" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="G10" s="49" t="s">
+      <c r="G10" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="H10" s="49" t="s">
+      <c r="H10" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="K10" s="37"/>
-      <c r="L10" s="38"/>
-      <c r="M10" s="38"/>
-      <c r="N10" s="39"/>
-      <c r="O10" s="39"/>
-      <c r="P10" s="40"/>
+      <c r="K10" s="52"/>
+      <c r="L10" s="53"/>
+      <c r="M10" s="53"/>
+      <c r="N10" s="56"/>
+      <c r="O10" s="56"/>
+      <c r="P10" s="57"/>
     </row>
     <row r="11" spans="2:24" ht="67.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B11" s="47" t="s">
+      <c r="B11" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="C11" s="48" t="s">
+      <c r="C11" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="D11" s="49" t="s">
+      <c r="D11" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="E11" s="49" t="s">
+      <c r="E11" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="F11" s="49" t="s">
+      <c r="F11" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="G11" s="49" t="s">
+      <c r="G11" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="H11" s="49" t="s">
+      <c r="H11" s="25" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="12" spans="2:24" ht="67.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B12" s="47" t="s">
+      <c r="B12" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="48" t="s">
+      <c r="C12" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="D12" s="49" t="s">
+      <c r="D12" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="E12" s="49" t="s">
+      <c r="E12" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="F12" s="49" t="s">
+      <c r="F12" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="G12" s="49" t="s">
+      <c r="G12" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="H12" s="49" t="s">
+      <c r="H12" s="25" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="13" spans="2:24" ht="67.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B13" s="47" t="s">
+      <c r="B13" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="C13" s="48" t="s">
+      <c r="C13" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="D13" s="49" t="s">
+      <c r="D13" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="E13" s="49" t="s">
+      <c r="E13" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="F13" s="49" t="s">
+      <c r="F13" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="G13" s="49" t="s">
+      <c r="G13" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="H13" s="49" t="s">
+      <c r="H13" s="25" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="14" spans="2:24" ht="67.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B14" s="50" t="s">
+      <c r="B14" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="C14" s="51" t="s">
+      <c r="C14" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="D14" s="52" t="s">
+      <c r="D14" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="E14" s="52" t="s">
+      <c r="E14" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="F14" s="52" t="s">
+      <c r="F14" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="G14" s="52" t="s">
+      <c r="G14" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="H14" s="52" t="s">
+      <c r="H14" s="28" t="s">
         <v>5</v>
       </c>
       <c r="I14" s="4"/>
@@ -5098,7 +4985,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="B1:X983"/>
+  <dimension ref="A1:X981"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="4.77734375" style="2" customWidth="1"/>
@@ -5114,16 +5001,16 @@
     <col min="18" max="16384" width="12.6640625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:24" ht="52.05" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B1" s="18" t="s">
+    <row r="1" spans="1:24" ht="52.05" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B1" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
     </row>
-    <row r="2" spans="2:24" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
@@ -5131,21 +5018,21 @@
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
     </row>
-    <row r="3" spans="2:24" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
     </row>
-    <row r="4" spans="2:24" s="11" customFormat="1" ht="76.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="20" t="s">
+    <row r="4" spans="1:24" s="11" customFormat="1" ht="76.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="46" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="20"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="46"/>
+      <c r="F4" s="46"/>
+      <c r="G4" s="46"/>
       <c r="J4" s="12"/>
       <c r="K4" s="12"/>
       <c r="L4" s="12"/>
@@ -5155,13 +5042,15 @@
       <c r="P4" s="12"/>
       <c r="Q4" s="12"/>
     </row>
-    <row r="5" spans="2:24" s="11" customFormat="1" ht="76.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="17"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
+    <row r="5" spans="1:24" s="11" customFormat="1" ht="76.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="77"/>
+      <c r="B5" s="78"/>
+      <c r="C5" s="78"/>
+      <c r="D5" s="78"/>
+      <c r="E5" s="78"/>
+      <c r="F5" s="78"/>
+      <c r="G5" s="78"/>
+      <c r="H5" s="77"/>
       <c r="J5" s="12"/>
       <c r="K5" s="12"/>
       <c r="L5" s="12"/>
@@ -5171,20 +5060,21 @@
       <c r="P5" s="12"/>
       <c r="Q5" s="12"/>
     </row>
-    <row r="6" spans="2:24" s="11" customFormat="1" ht="69" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="67" t="s">
+    <row r="6" spans="1:24" s="11" customFormat="1" ht="69" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="77"/>
+      <c r="B6" s="69" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="71" t="s">
+      <c r="C6" s="67" t="s">
         <v>53</v>
       </c>
-      <c r="D6" s="72"/>
-      <c r="E6" s="71" t="s">
+      <c r="D6" s="68"/>
+      <c r="E6" s="67" t="s">
         <v>54</v>
       </c>
-      <c r="F6" s="73"/>
-      <c r="G6" s="72"/>
-      <c r="H6" s="74" t="s">
+      <c r="F6" s="71"/>
+      <c r="G6" s="68"/>
+      <c r="H6" s="37" t="s">
         <v>55</v>
       </c>
       <c r="J6" s="12"/>
@@ -5196,238 +5086,253 @@
       <c r="P6" s="12"/>
       <c r="Q6" s="12"/>
     </row>
-    <row r="7" spans="2:24" ht="67.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B7" s="68"/>
-      <c r="C7" s="69" t="s">
+    <row r="7" spans="1:24" ht="67.95" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="79"/>
+      <c r="B7" s="70"/>
+      <c r="C7" s="35" t="s">
         <v>33</v>
       </c>
-      <c r="D7" s="69" t="s">
+      <c r="D7" s="35" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="70" t="s">
+      <c r="E7" s="36" t="s">
         <v>27</v>
       </c>
-      <c r="F7" s="70" t="s">
+      <c r="F7" s="36" t="s">
         <v>28</v>
       </c>
-      <c r="G7" s="70" t="s">
+      <c r="G7" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="H7" s="66" t="s">
+      <c r="H7" s="34" t="s">
         <v>31</v>
       </c>
-      <c r="K7" s="21" t="s">
+      <c r="K7" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="L7" s="22"/>
-      <c r="M7" s="22"/>
-      <c r="N7" s="22"/>
-      <c r="O7" s="22"/>
-      <c r="P7" s="23"/>
+      <c r="L7" s="48"/>
+      <c r="M7" s="48"/>
+      <c r="N7" s="48"/>
+      <c r="O7" s="48"/>
+      <c r="P7" s="49"/>
     </row>
-    <row r="8" spans="2:24" ht="49.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B8" s="65" t="s">
+    <row r="8" spans="1:24" ht="49.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="79"/>
+      <c r="B8" s="33" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="62" t="s">
+      <c r="C8" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="D8" s="62" t="s">
+      <c r="D8" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="E8" s="63"/>
-      <c r="F8" s="62" t="s">
+      <c r="E8" s="32"/>
+      <c r="F8" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="G8" s="62" t="s">
+      <c r="G8" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="H8" s="62"/>
-      <c r="K8" s="55" t="s">
+      <c r="H8" s="32"/>
+      <c r="K8" s="40" t="s">
         <v>49</v>
       </c>
-      <c r="L8" s="55"/>
-      <c r="M8" s="55"/>
-      <c r="N8" s="56" t="s">
+      <c r="L8" s="40"/>
+      <c r="M8" s="40"/>
+      <c r="N8" s="42" t="s">
         <v>50</v>
       </c>
-      <c r="O8" s="56"/>
-      <c r="P8" s="56"/>
+      <c r="O8" s="42"/>
+      <c r="P8" s="42"/>
     </row>
-    <row r="9" spans="2:24" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B9" s="65" t="s">
+    <row r="9" spans="1:24" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="79"/>
+      <c r="B9" s="33" t="s">
         <v>35</v>
       </c>
-      <c r="C9" s="62" t="s">
+      <c r="C9" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="D9" s="63"/>
-      <c r="E9" s="62" t="s">
+      <c r="D9" s="32"/>
+      <c r="E9" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="F9" s="62" t="s">
+      <c r="F9" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="G9" s="62" t="s">
+      <c r="G9" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="H9" s="62"/>
-      <c r="K9" s="57"/>
-      <c r="L9" s="57"/>
-      <c r="M9" s="57"/>
-      <c r="N9" s="58"/>
-      <c r="O9" s="58"/>
-      <c r="P9" s="58"/>
+      <c r="H9" s="32"/>
+      <c r="K9" s="41"/>
+      <c r="L9" s="41"/>
+      <c r="M9" s="41"/>
+      <c r="N9" s="43"/>
+      <c r="O9" s="43"/>
+      <c r="P9" s="43"/>
     </row>
-    <row r="10" spans="2:24" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B10" s="65" t="s">
+    <row r="10" spans="1:24" ht="46.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="79"/>
+      <c r="B10" s="33" t="s">
         <v>36</v>
       </c>
-      <c r="C10" s="62" t="s">
+      <c r="C10" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="D10" s="62" t="s">
+      <c r="D10" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="E10" s="62" t="s">
+      <c r="E10" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="F10" s="63"/>
-      <c r="G10" s="62" t="s">
+      <c r="F10" s="32"/>
+      <c r="G10" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="H10" s="62"/>
-      <c r="K10" s="57"/>
-      <c r="L10" s="57"/>
-      <c r="M10" s="57"/>
-      <c r="N10" s="58"/>
-      <c r="O10" s="58"/>
-      <c r="P10" s="58"/>
+      <c r="H10" s="32"/>
+      <c r="K10" s="41"/>
+      <c r="L10" s="41"/>
+      <c r="M10" s="41"/>
+      <c r="N10" s="43"/>
+      <c r="O10" s="43"/>
+      <c r="P10" s="43"/>
     </row>
-    <row r="11" spans="2:24" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B11" s="65" t="s">
+    <row r="11" spans="1:24" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="79"/>
+      <c r="B11" s="33" t="s">
         <v>37</v>
       </c>
-      <c r="C11" s="63"/>
-      <c r="D11" s="62" t="s">
+      <c r="C11" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="E11" s="62" t="s">
+      <c r="D11" s="32" t="s">
+        <v>4</v>
+      </c>
+      <c r="E11" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="F11" s="63"/>
-      <c r="G11" s="63"/>
-      <c r="H11" s="62"/>
-      <c r="K11" s="57"/>
-      <c r="L11" s="57"/>
-      <c r="M11" s="57"/>
-      <c r="N11" s="58"/>
-      <c r="O11" s="58"/>
-      <c r="P11" s="58"/>
+      <c r="F11" s="32"/>
+      <c r="G11" s="32"/>
+      <c r="H11" s="32"/>
+      <c r="K11" s="41"/>
+      <c r="L11" s="41"/>
+      <c r="M11" s="41"/>
+      <c r="N11" s="43"/>
+      <c r="O11" s="43"/>
+      <c r="P11" s="43"/>
     </row>
-    <row r="12" spans="2:24" ht="38.4" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B12" s="65" t="s">
+    <row r="12" spans="1:24" ht="38.4" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="79"/>
+      <c r="B12" s="33" t="s">
         <v>38</v>
       </c>
-      <c r="C12" s="62" t="s">
+      <c r="C12" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="D12" s="72" t="s">
+        <v>2</v>
+      </c>
+      <c r="E12" s="32" t="s">
+        <v>4</v>
+      </c>
+      <c r="F12" s="32" t="s">
+        <v>2</v>
+      </c>
+      <c r="G12" s="32"/>
+      <c r="H12" s="32"/>
+      <c r="K12" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="L12" s="38"/>
+      <c r="M12" s="38"/>
+      <c r="N12" s="39" t="s">
+        <v>52</v>
+      </c>
+      <c r="O12" s="39"/>
+      <c r="P12" s="39"/>
+    </row>
+    <row r="13" spans="1:24" ht="30.6" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="79"/>
+      <c r="B13" s="33" t="s">
+        <v>39</v>
+      </c>
+      <c r="C13" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="D13" s="32" t="s">
+        <v>2</v>
+      </c>
+      <c r="E13" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="D12" s="64"/>
-      <c r="E12" s="62" t="s">
+      <c r="F13" s="32" t="s">
+        <v>5</v>
+      </c>
+      <c r="G13" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="F12" s="62" t="s">
+      <c r="H13" s="32"/>
+      <c r="K13" s="38"/>
+      <c r="L13" s="38"/>
+      <c r="M13" s="38"/>
+      <c r="N13" s="39"/>
+      <c r="O13" s="39"/>
+      <c r="P13" s="39"/>
+    </row>
+    <row r="14" spans="1:24" ht="43.8" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="79"/>
+      <c r="B14" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="G12" s="63"/>
-      <c r="H12" s="62"/>
-      <c r="K12" s="59" t="s">
-        <v>51</v>
-      </c>
-      <c r="L12" s="59"/>
-      <c r="M12" s="59"/>
-      <c r="N12" s="60" t="s">
-        <v>52</v>
-      </c>
-      <c r="O12" s="60"/>
-      <c r="P12" s="60"/>
+      <c r="D14" s="32" t="s">
+        <v>4</v>
+      </c>
+      <c r="E14" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="F14" s="32" t="s">
+        <v>2</v>
+      </c>
+      <c r="G14" s="32"/>
+      <c r="H14" s="32"/>
+      <c r="K14" s="38"/>
+      <c r="L14" s="38"/>
+      <c r="M14" s="38"/>
+      <c r="N14" s="39"/>
+      <c r="O14" s="39"/>
+      <c r="P14" s="39"/>
     </row>
-    <row r="13" spans="2:24" ht="30.6" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B13" s="65" t="s">
-        <v>39</v>
-      </c>
-      <c r="C13" s="62" t="s">
+    <row r="15" spans="1:24" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="79"/>
+      <c r="B15" s="33" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" s="32"/>
+      <c r="D15" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="D13" s="62" t="s">
-        <v>3</v>
-      </c>
-      <c r="E13" s="63"/>
-      <c r="F13" s="62" t="s">
-        <v>5</v>
-      </c>
-      <c r="G13" s="62" t="s">
+      <c r="E15" s="32" t="s">
+        <v>2</v>
+      </c>
+      <c r="F15" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="H13" s="62"/>
-      <c r="K13" s="59"/>
-      <c r="L13" s="59"/>
-      <c r="M13" s="59"/>
-      <c r="N13" s="60"/>
-      <c r="O13" s="60"/>
-      <c r="P13" s="60"/>
-    </row>
-    <row r="14" spans="2:24" ht="43.8" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B14" s="65" t="s">
-        <v>40</v>
-      </c>
-      <c r="C14" s="62" t="s">
-        <v>2</v>
-      </c>
-      <c r="D14" s="62" t="s">
-        <v>4</v>
-      </c>
-      <c r="E14" s="62" t="s">
-        <v>3</v>
-      </c>
-      <c r="F14" s="62" t="s">
-        <v>2</v>
-      </c>
-      <c r="G14" s="63"/>
-      <c r="H14" s="62"/>
-      <c r="K14" s="59"/>
-      <c r="L14" s="59"/>
-      <c r="M14" s="59"/>
-      <c r="N14" s="60"/>
-      <c r="O14" s="60"/>
-      <c r="P14" s="60"/>
-    </row>
-    <row r="15" spans="2:24" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="65" t="s">
-        <v>41</v>
-      </c>
-      <c r="C15" s="63"/>
-      <c r="D15" s="62" t="s">
-        <v>2</v>
-      </c>
-      <c r="E15" s="62" t="s">
-        <v>2</v>
-      </c>
-      <c r="F15" s="62" t="s">
-        <v>4</v>
-      </c>
-      <c r="G15" s="63"/>
-      <c r="H15" s="62" t="s">
+      <c r="G15" s="32"/>
+      <c r="H15" s="32" t="s">
         <v>5</v>
       </c>
       <c r="I15" s="4"/>
       <c r="J15" s="10"/>
-      <c r="K15" s="59"/>
-      <c r="L15" s="59"/>
-      <c r="M15" s="59"/>
-      <c r="N15" s="60"/>
-      <c r="O15" s="60"/>
-      <c r="P15" s="60"/>
+      <c r="K15" s="38"/>
+      <c r="L15" s="38"/>
+      <c r="M15" s="38"/>
+      <c r="N15" s="39"/>
+      <c r="O15" s="39"/>
+      <c r="P15" s="39"/>
       <c r="Q15" s="10"/>
       <c r="R15" s="4"/>
       <c r="S15" s="4"/>
@@ -5437,34 +5342,37 @@
       <c r="W15" s="4"/>
       <c r="X15" s="4"/>
     </row>
-    <row r="16" spans="2:24" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="65" t="s">
+    <row r="16" spans="1:24" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="79"/>
+      <c r="B16" s="33" t="s">
         <v>42</v>
       </c>
-      <c r="C16" s="62" t="s">
+      <c r="C16" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="D16" s="32" t="s">
+        <v>4</v>
+      </c>
+      <c r="E16" s="32" t="s">
+        <v>5</v>
+      </c>
+      <c r="F16" s="32" t="s">
+        <v>5</v>
+      </c>
+      <c r="G16" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="D16" s="62" t="s">
-        <v>4</v>
-      </c>
-      <c r="E16" s="62" t="s">
-        <v>5</v>
-      </c>
-      <c r="F16" s="62" t="s">
-        <v>5</v>
-      </c>
-      <c r="G16" s="62" t="s">
+      <c r="H16" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="H16" s="62"/>
       <c r="I16" s="4"/>
       <c r="J16" s="10"/>
-      <c r="K16" s="59"/>
-      <c r="L16" s="59"/>
-      <c r="M16" s="59"/>
-      <c r="N16" s="60"/>
-      <c r="O16" s="60"/>
-      <c r="P16" s="60"/>
+      <c r="K16" s="38"/>
+      <c r="L16" s="38"/>
+      <c r="M16" s="38"/>
+      <c r="N16" s="39"/>
+      <c r="O16" s="39"/>
+      <c r="P16" s="39"/>
       <c r="Q16" s="10"/>
       <c r="R16" s="4"/>
       <c r="S16" s="4"/>
@@ -5474,34 +5382,35 @@
       <c r="W16" s="4"/>
       <c r="X16" s="4"/>
     </row>
-    <row r="17" spans="2:24" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="65" t="s">
+    <row r="17" spans="1:24" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="79"/>
+      <c r="B17" s="33" t="s">
         <v>43</v>
       </c>
-      <c r="C17" s="62" t="s">
+      <c r="C17" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="D17" s="62" t="s">
+      <c r="D17" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="E17" s="62" t="s">
+      <c r="E17" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="F17" s="62" t="s">
+      <c r="F17" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="G17" s="62" t="s">
+      <c r="G17" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="H17" s="62"/>
+      <c r="H17" s="32"/>
       <c r="I17" s="4"/>
       <c r="J17" s="10"/>
-      <c r="K17" s="59"/>
-      <c r="L17" s="59"/>
-      <c r="M17" s="59"/>
-      <c r="N17" s="60"/>
-      <c r="O17" s="60"/>
-      <c r="P17" s="60"/>
+      <c r="K17" s="38"/>
+      <c r="L17" s="38"/>
+      <c r="M17" s="38"/>
+      <c r="N17" s="39"/>
+      <c r="O17" s="39"/>
+      <c r="P17" s="39"/>
       <c r="Q17" s="10"/>
       <c r="R17" s="4"/>
       <c r="S17" s="4"/>
@@ -5511,28 +5420,64 @@
       <c r="W17" s="4"/>
       <c r="X17" s="4"/>
     </row>
-    <row r="18" spans="2:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="K18" s="59"/>
-      <c r="L18" s="59"/>
-      <c r="M18" s="59"/>
-      <c r="N18" s="60"/>
-      <c r="O18" s="60"/>
-      <c r="P18" s="60"/>
+    <row r="18" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="79"/>
+      <c r="B18" s="79"/>
+      <c r="C18" s="79"/>
+      <c r="D18" s="79"/>
+      <c r="E18" s="79"/>
+      <c r="F18" s="79"/>
+      <c r="G18" s="80"/>
+      <c r="H18" s="79"/>
     </row>
-    <row r="19" spans="2:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="20" spans="2:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="21" spans="2:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="22" spans="2:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="23" spans="2:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="24" spans="2:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="25" spans="2:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="26" spans="2:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="27" spans="2:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="28" spans="2:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="29" spans="2:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="30" spans="2:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="31" spans="2:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="32" spans="2:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="19" spans="1:24" ht="6" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="79"/>
+      <c r="B19" s="79"/>
+      <c r="C19" s="79"/>
+      <c r="D19" s="79"/>
+      <c r="E19" s="79"/>
+      <c r="F19" s="79"/>
+      <c r="G19" s="81"/>
+      <c r="H19" s="79"/>
+    </row>
+    <row r="20" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="79"/>
+      <c r="B20" s="79"/>
+      <c r="C20" s="73" t="s">
+        <v>56</v>
+      </c>
+      <c r="D20" s="74" t="s">
+        <v>57</v>
+      </c>
+      <c r="E20" s="75" t="s">
+        <v>58</v>
+      </c>
+      <c r="F20" s="76" t="s">
+        <v>59</v>
+      </c>
+      <c r="G20" s="79"/>
+      <c r="H20" s="79"/>
+    </row>
+    <row r="21" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B21" s="79"/>
+      <c r="C21" s="73"/>
+      <c r="D21" s="74"/>
+      <c r="E21" s="75"/>
+      <c r="F21" s="76"/>
+      <c r="G21" s="79"/>
+      <c r="H21" s="79"/>
+    </row>
+    <row r="22" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="23" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="24" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="25" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="26" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="27" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="28" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="29" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="30" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="31" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="32" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
     <row r="33" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
     <row r="34" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
     <row r="35" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
@@ -6482,20 +6427,23 @@
     <row r="979" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
     <row r="980" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
     <row r="981" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="982" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="983" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="15">
+    <mergeCell ref="G18:G19"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="E20:E21"/>
+    <mergeCell ref="F20:F21"/>
+    <mergeCell ref="K12:M17"/>
+    <mergeCell ref="N12:P17"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="E6:G6"/>
     <mergeCell ref="B1:F1"/>
     <mergeCell ref="B4:G4"/>
     <mergeCell ref="K7:P7"/>
     <mergeCell ref="K8:M11"/>
     <mergeCell ref="N8:P11"/>
-    <mergeCell ref="K12:M18"/>
-    <mergeCell ref="N12:P18"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="E6:G6"/>
   </mergeCells>
   <conditionalFormatting sqref="C8:H17">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">

</xml_diff>